<commit_message>
hemogen pack 번역 갱신
</commit_message>
<xml_diff>
--- a/Data/AOBA/Hemogen Pack - Emergency transfusion - 3778942862/Hemogen Pack - Emergency transfusion - 3778942862.xlsx
+++ b/Data/AOBA/Hemogen Pack - Emergency transfusion - 3778942862/Hemogen Pack - Emergency transfusion - 3778942862.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="32">
   <si>
     <t xml:space="preserve">Class+Node [(Identifier (Key)]</t>
   </si>
@@ -66,7 +66,7 @@
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Segoe UI"/>
+        <rFont val="맑은 고딕"/>
         <family val="2"/>
         <charset val="129"/>
       </rPr>
@@ -86,7 +86,7 @@
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Segoe UI"/>
+        <rFont val="맑은 고딕"/>
         <family val="2"/>
         <charset val="129"/>
       </rPr>
@@ -94,6 +94,53 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">Patches.ThingDef+HemogenPack.comps.1.useLabel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patches.ThingDef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HemogenPack.comps.1.useLabel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biotech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administer {0_label}...</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">{0_label} </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">수혈</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">... </t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">Keyed+HD_UseHemogenPackLabel</t>
   </si>
   <si>
@@ -103,108 +150,73 @@
     <t xml:space="preserve">HD_UseHemogenPackLabel</t>
   </si>
   <si>
-    <t xml:space="preserve">Administer {0_label}...</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">{0_label} </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Segoe UI"/>
+    <t xml:space="preserve">Keyed+HD_MessageCannotReach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HD_MessageCannotReach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{0} cannot reach {1}.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">{0}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
         <family val="2"/>
         <charset val="129"/>
       </rPr>
-      <t xml:space="preserve">수혈</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">... </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Keyed+HD_MessageCannotReach</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HD_MessageCannotReach</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{0} cannot reach {1}.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">{0}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Segoe UI"/>
+      <t xml:space="preserve">은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
         <family val="2"/>
         <charset val="129"/>
       </rPr>
-      <t xml:space="preserve">은</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Segoe UI"/>
+      <t xml:space="preserve">는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">) {1}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
         <family val="2"/>
         <charset val="129"/>
       </rPr>
-      <t xml:space="preserve">는</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">) {1}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Segoe UI"/>
-        <family val="2"/>
-        <charset val="129"/>
-      </rPr>
       <t xml:space="preserve">에 도달할 수 없습니다</t>
     </r>
     <r>
@@ -244,7 +256,7 @@
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Segoe UI"/>
+        <rFont val="맑은 고딕"/>
         <family val="2"/>
         <charset val="129"/>
       </rPr>
@@ -269,7 +281,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -312,14 +324,7 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-      <charset val="129"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Segoe UI"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <charset val="129"/>
     </font>
@@ -366,20 +371,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -579,15 +588,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultColWidth="8.390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="1" style="1" width="8.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="38.78"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="68.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="54.97"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="8.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="45.92"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="8.39"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -607,7 +619,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -623,8 +635,9 @@
       <c r="F2" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="G2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -634,36 +647,41 @@
       <c r="C3" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="D3" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="E3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="F4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>21</v>
@@ -671,16 +689,17 @@
       <c r="E5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>23</v>
       </c>
+      <c r="G5" s="3"/>
     </row>
-    <row r="6" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>25</v>
@@ -691,6 +710,25 @@
       <c r="F6" s="4" t="s">
         <v>27</v>
       </c>
+      <c r="G6" s="3"/>
+    </row>
+    <row r="7" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>